<commit_message>
feat: add the OCR + LLM as a fallback when API request fails and do some evaluation towards the VLM result
</commit_message>
<xml_diff>
--- a/data/ground_truth/ARCI.xlsx
+++ b/data/ground_truth/ARCI.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadnajmirahmani/Belajar/ProjectDatasaur/data/ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{28F611F0-C951-8544-BE6B-D57EF0C34737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A02C08A-CDC6-E84B-9040-C2905D8A04C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29300" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="lokasi kebun" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="lokasi kebun" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="71">
   <si>
     <t>Perusahaan</t>
   </si>
@@ -54,9 +55,6 @@
     <t>PT Cipta Davia Mandiri</t>
   </si>
   <si>
-    <t>TLDN</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kutai Timur, Kaltim </t>
   </si>
   <si>
@@ -238,18 +236,34 @@
   </si>
   <si>
     <t>DER</t>
+  </si>
+  <si>
+    <t>ARCI</t>
+  </si>
+  <si>
+    <t>Kurs</t>
+  </si>
+  <si>
+    <t>USD to IDR</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Converted</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +283,24 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -296,10 +328,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -329,8 +362,15 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -556,15 +596,24 @@
     <col min="9" max="9" width="19.5" customWidth="1"/>
     <col min="10" max="10" width="17.5" customWidth="1"/>
     <col min="11" max="11" width="17.1640625" customWidth="1"/>
-    <col min="12" max="27" width="8.6640625" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="8.6640625" customWidth="1"/>
+    <col min="16" max="16" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="32.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15" bestFit="1" customWidth="1"/>
+    <col min="21" max="23" width="8.6640625" customWidth="1"/>
+    <col min="24" max="24" width="15" bestFit="1" customWidth="1"/>
+    <col min="25" max="27" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>5</v>
+      <c r="D1" s="15" t="s">
+        <v>66</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -591,12 +640,12 @@
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -622,124 +671,114 @@
     <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="6" t="s">
+      <c r="T3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="U3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="U3" s="6" t="s">
+      <c r="V3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="V3" s="6" t="s">
+      <c r="W3" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="X3" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="Y3" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="Z3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="Z3" s="6" t="s">
+      <c r="AA3" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="AA3" s="6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="7">
-        <v>6342799138000</v>
-      </c>
-      <c r="C4" s="7">
-        <v>6287074631000</v>
-      </c>
-      <c r="D4" s="7">
-        <v>6018032137000</v>
-      </c>
-      <c r="E4" s="7">
-        <v>6207108405000</v>
-      </c>
-      <c r="F4" s="7">
-        <v>5922715715000</v>
-      </c>
-      <c r="G4" s="7">
-        <v>5976239681000</v>
-      </c>
-      <c r="H4" s="7">
-        <v>5664445219000</v>
-      </c>
-      <c r="I4" s="7">
-        <v>5436056871000</v>
-      </c>
-      <c r="J4" s="7">
-        <v>5171540190000</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
       <c r="M4" s="5"/>
       <c r="N4" s="8"/>
       <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
+      <c r="P4" s="8">
+        <v>11286421729559.748</v>
+      </c>
+      <c r="Q4" s="16">
+        <v>11028397774390.242</v>
+      </c>
+      <c r="R4" s="5">
+        <v>10560298900445.766</v>
+      </c>
+      <c r="S4" s="5">
+        <v>9966590200860.832</v>
+      </c>
       <c r="T4" s="5"/>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
@@ -751,44 +790,34 @@
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="7">
-        <v>1914357059000</v>
-      </c>
-      <c r="C5" s="7">
-        <v>1952459070000</v>
-      </c>
-      <c r="D5" s="7">
-        <v>1588829853000</v>
-      </c>
-      <c r="E5" s="7">
-        <v>1819609212000</v>
-      </c>
-      <c r="F5" s="7">
-        <v>1684520584000</v>
-      </c>
-      <c r="G5" s="7">
-        <v>2073151943000</v>
-      </c>
-      <c r="H5" s="7">
-        <v>1766579819000</v>
-      </c>
-      <c r="I5" s="7">
-        <v>1702439782000</v>
-      </c>
-      <c r="J5" s="7">
-        <v>1596650258000</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="5"/>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
+      <c r="P5" s="6">
+        <v>1370668490566.0376</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>1142124496951.2195</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1296301263001.4858</v>
+      </c>
+      <c r="S5" s="5">
+        <v>1052012410329.9857</v>
+      </c>
       <c r="T5" s="5"/>
       <c r="U5" s="9"/>
       <c r="V5" s="9"/>
@@ -800,44 +829,34 @@
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="7">
-        <v>258018162000</v>
-      </c>
-      <c r="C6" s="7">
-        <v>695168978000</v>
-      </c>
-      <c r="D6" s="7">
-        <v>334385754000</v>
-      </c>
-      <c r="E6" s="7">
-        <v>453355101000</v>
-      </c>
-      <c r="F6" s="7">
-        <v>276683736000</v>
-      </c>
-      <c r="G6" s="7">
-        <v>821851671000</v>
-      </c>
-      <c r="H6" s="7">
-        <v>486587666000</v>
-      </c>
-      <c r="I6" s="7">
-        <v>506251051000</v>
-      </c>
-      <c r="J6" s="7">
-        <v>380517170000</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
       <c r="K6" s="8"/>
       <c r="L6" s="8"/>
       <c r="M6" s="5"/>
       <c r="N6" s="6"/>
       <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
+      <c r="P6" s="8">
+        <v>162569716981.13208</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>146141859756.09753</v>
+      </c>
+      <c r="R6" s="20">
+        <v>184978038633</v>
+      </c>
+      <c r="S6" s="5">
+        <v>331786255380.20087</v>
+      </c>
       <c r="T6" s="5"/>
       <c r="U6" s="9"/>
       <c r="V6" s="9"/>
@@ -849,44 +868,34 @@
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="7">
-        <v>2651152175000</v>
-      </c>
-      <c r="C7" s="7">
-        <v>2460394233000</v>
-      </c>
-      <c r="D7" s="7">
-        <v>2373123326000</v>
-      </c>
-      <c r="E7" s="7">
-        <v>2631574846000</v>
-      </c>
-      <c r="F7" s="7">
-        <v>2615212576000</v>
-      </c>
-      <c r="G7" s="7">
-        <v>2612501553000</v>
-      </c>
-      <c r="H7" s="7">
-        <v>2519627219000</v>
-      </c>
-      <c r="I7" s="7">
-        <v>3196613547000</v>
-      </c>
-      <c r="J7" s="10">
-        <v>3102894029000</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="10"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
       <c r="M7" s="5"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="5"/>
+      <c r="P7" s="8">
+        <v>7390895959119</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>7248177850609.7549</v>
+      </c>
+      <c r="R7" s="16">
+        <v>6892214918276.375</v>
+      </c>
+      <c r="S7" s="5">
+        <v>6491908593974.1758</v>
+      </c>
       <c r="T7" s="5"/>
       <c r="U7" s="9"/>
       <c r="V7" s="9"/>
@@ -898,46 +907,34 @@
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="7">
-        <v>124347189000</v>
-      </c>
-      <c r="C8" s="7">
-        <v>165863709000</v>
-      </c>
-      <c r="D8" s="7">
-        <v>190767674000</v>
-      </c>
-      <c r="E8" s="7">
-        <v>141500000000</v>
-      </c>
-      <c r="F8" s="7">
-        <v>122902518000</v>
-      </c>
-      <c r="G8" s="7">
-        <v>290757191000</v>
-      </c>
-      <c r="H8" s="5">
-        <f>20000000000+337603441000</f>
-        <v>357603441000</v>
-      </c>
-      <c r="I8" s="5">
-        <f>441100000000</f>
-        <v>441100000000</v>
-      </c>
-      <c r="J8" s="10">
-        <v>469775000000</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="10"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="5"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="5"/>
+      <c r="P8" s="8">
+        <v>1503778443396</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>1221905746951.2192</v>
+      </c>
+      <c r="R8" s="5">
+        <v>959718053491.82776</v>
+      </c>
+      <c r="S8" s="5">
+        <v>1468543529411.7646</v>
+      </c>
       <c r="T8" s="5"/>
       <c r="U8" s="9"/>
       <c r="V8" s="9"/>
@@ -949,44 +946,34 @@
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="7">
-        <v>3691598827000</v>
-      </c>
-      <c r="C9" s="7">
-        <v>3826634977000</v>
-      </c>
-      <c r="D9" s="7">
-        <v>3644864762000</v>
-      </c>
-      <c r="E9" s="7">
-        <v>3575485566000</v>
-      </c>
-      <c r="F9" s="7">
-        <v>3307456949000</v>
-      </c>
-      <c r="G9" s="7">
-        <v>3363694421000</v>
-      </c>
-      <c r="H9" s="7">
-        <v>3144775624000</v>
-      </c>
-      <c r="I9" s="7">
-        <v>2239409582000</v>
-      </c>
-      <c r="J9" s="10">
-        <v>2068614365000</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="10"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
       <c r="M9" s="5"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
+      <c r="P9" s="8">
+        <v>3896822720126</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>3782433124999.9995</v>
+      </c>
+      <c r="R9" s="16">
+        <v>3670567132243.6851</v>
+      </c>
+      <c r="S9" s="5">
+        <v>3475782496413.1997</v>
+      </c>
       <c r="T9" s="5"/>
       <c r="U9" s="9"/>
       <c r="V9" s="9"/>
@@ -998,44 +985,34 @@
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="7">
-        <v>543642277000</v>
-      </c>
-      <c r="C10" s="7">
-        <v>181770215000</v>
-      </c>
-      <c r="D10" s="7">
-        <v>1106606494000</v>
-      </c>
-      <c r="E10" s="7">
-        <v>829300009000</v>
-      </c>
-      <c r="F10" s="7">
-        <v>561271392000</v>
-      </c>
-      <c r="G10" s="7">
-        <v>218918797000</v>
-      </c>
-      <c r="H10" s="7">
-        <v>825587405000</v>
-      </c>
-      <c r="I10" s="7">
-        <v>234190360000</v>
-      </c>
-      <c r="J10" s="10">
-        <v>63395143000</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="10"/>
       <c r="K10" s="8"/>
       <c r="L10" s="5"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="5"/>
+      <c r="P10" s="8">
+        <v>228784339623</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>231810807926.82925</v>
+      </c>
+      <c r="R10" s="5">
+        <v>210274992570.5795</v>
+      </c>
+      <c r="S10" s="5">
+        <v>135587948350.07175</v>
+      </c>
       <c r="T10" s="5"/>
       <c r="U10" s="9"/>
       <c r="V10" s="9"/>
@@ -1047,44 +1024,34 @@
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="7">
-        <v>2968533550000</v>
-      </c>
-      <c r="C11" s="7">
-        <v>1587018948000</v>
-      </c>
-      <c r="D11" s="7">
-        <v>5330133466000</v>
-      </c>
-      <c r="E11" s="7">
-        <v>4028946553000</v>
-      </c>
-      <c r="F11" s="7">
-        <v>2691885302000</v>
-      </c>
-      <c r="G11" s="7">
-        <v>1457165917000</v>
-      </c>
-      <c r="H11" s="7">
-        <v>4211481582000</v>
-      </c>
-      <c r="I11" s="7">
-        <v>2885430562000</v>
-      </c>
-      <c r="J11" s="7">
-        <v>1915665661000</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
+      <c r="P11" s="5">
+        <v>3403714968553</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>2525081006097.5605</v>
+      </c>
+      <c r="R11" s="5">
+        <v>1777560772659.7327</v>
+      </c>
+      <c r="S11" s="5">
+        <v>1149631348637.0159</v>
+      </c>
       <c r="T11" s="5"/>
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
@@ -1096,44 +1063,34 @@
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="7">
-        <v>851671746000</v>
-      </c>
-      <c r="C12" s="7">
-        <v>545153215000</v>
-      </c>
-      <c r="D12" s="7">
-        <v>1544117069000</v>
-      </c>
-      <c r="E12" s="7">
-        <v>1670634109000</v>
-      </c>
-      <c r="F12" s="7">
-        <v>1199712765000</v>
-      </c>
-      <c r="G12" s="7">
-        <v>612102984000</v>
-      </c>
-      <c r="H12" s="7">
-        <v>1140257076000</v>
-      </c>
-      <c r="I12" s="7">
-        <v>947753157000</v>
-      </c>
-      <c r="J12" s="10">
-        <v>1901117155000</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="10"/>
       <c r="K12" s="8"/>
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="5"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
+      <c r="P12" s="8">
+        <v>853635345912</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>560685746951.21948</v>
+      </c>
+      <c r="R12" s="5">
+        <v>247243491827.63745</v>
+      </c>
+      <c r="S12" s="5">
+        <v>522079942611.19086</v>
+      </c>
       <c r="T12" s="5"/>
       <c r="U12" s="9"/>
       <c r="V12" s="9"/>
@@ -1145,44 +1102,34 @@
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="C13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="D13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="E13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="F13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="G13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="H13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="I13" s="7">
-        <v>12946530200</v>
-      </c>
-      <c r="J13" s="7">
-        <v>12946530200</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
+      <c r="P13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="R13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="S13" s="5">
+        <v>24835000000</v>
+      </c>
       <c r="T13" s="5"/>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
@@ -1194,35 +1141,17 @@
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="4">
-        <v>555</v>
-      </c>
-      <c r="C14" s="4">
-        <v>472</v>
-      </c>
-      <c r="D14" s="4">
-        <v>600</v>
-      </c>
-      <c r="E14" s="4">
-        <v>715</v>
-      </c>
-      <c r="F14" s="4">
-        <v>630</v>
-      </c>
-      <c r="G14" s="4">
-        <v>580</v>
-      </c>
-      <c r="H14" s="5">
-        <v>585</v>
-      </c>
-      <c r="I14" s="5">
-        <v>520</v>
-      </c>
-      <c r="J14" s="5">
-        <v>462</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
       <c r="K14" s="5">
         <v>444</v>
       </c>
@@ -1248,7 +1177,7 @@
         <v>610</v>
       </c>
       <c r="S14" s="5">
-        <v>650</v>
+        <v>352</v>
       </c>
       <c r="T14" s="5">
         <v>725</v>
@@ -1277,43 +1206,43 @@
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="6">
+        <v>58</v>
+      </c>
+      <c r="B15" s="6" t="e">
         <f t="shared" ref="B15:AA15" si="0">B9/B13</f>
-        <v>285.14194691331272</v>
-      </c>
-      <c r="C15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>295.5722435189623</v>
-      </c>
-      <c r="D15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>281.53217160842058</v>
-      </c>
-      <c r="E15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>276.17326888095471</v>
-      </c>
-      <c r="F15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>255.47053132429258</v>
-      </c>
-      <c r="G15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>259.81435713176649</v>
-      </c>
-      <c r="H15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>242.90490003259714</v>
-      </c>
-      <c r="I15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>172.97372712265405</v>
-      </c>
-      <c r="J15" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J15" s="6" t="e">
         <f t="shared" si="0"/>
-        <v>159.78137254103805</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K15" s="6" t="e">
         <f t="shared" si="0"/>
@@ -1335,21 +1264,21 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P15" s="6" t="e">
+      <c r="P15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q15" s="6" t="e">
+        <v>156.90850493762835</v>
+      </c>
+      <c r="Q15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R15" s="6" t="e">
+        <v>152.30252164284275</v>
+      </c>
+      <c r="R15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S15" s="6" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>147.79815310020879</v>
+      </c>
+      <c r="S15" s="6">
+        <f>S9/S13</f>
+        <v>139.95500287550632</v>
       </c>
       <c r="T15" s="6" t="e">
         <f t="shared" si="0"/>
@@ -1386,43 +1315,43 @@
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B16" s="6">
         <f t="shared" ref="B16:AA16" si="1">B5-B7</f>
-        <v>-736795116000</v>
+        <v>0</v>
       </c>
       <c r="C16" s="6">
         <f t="shared" si="1"/>
-        <v>-507935163000</v>
+        <v>0</v>
       </c>
       <c r="D16" s="6">
         <f t="shared" si="1"/>
-        <v>-784293473000</v>
+        <v>0</v>
       </c>
       <c r="E16" s="6">
         <f t="shared" si="1"/>
-        <v>-811965634000</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6">
         <f t="shared" si="1"/>
-        <v>-930691992000</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6">
         <f t="shared" si="1"/>
-        <v>-539349610000</v>
+        <v>0</v>
       </c>
       <c r="H16" s="6">
         <f t="shared" si="1"/>
-        <v>-753047400000</v>
+        <v>0</v>
       </c>
       <c r="I16" s="6">
         <f t="shared" si="1"/>
-        <v>-1494173765000</v>
+        <v>0</v>
       </c>
       <c r="J16" s="6">
         <f t="shared" si="1"/>
-        <v>-1506243771000</v>
+        <v>0</v>
       </c>
       <c r="K16" s="6">
         <f t="shared" si="1"/>
@@ -1446,19 +1375,19 @@
       </c>
       <c r="P16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6020227468552.9629</v>
       </c>
       <c r="Q16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6106053353658.5352</v>
       </c>
       <c r="R16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-5595913655274.8887</v>
       </c>
       <c r="S16" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>S5-S7</f>
+        <v>-5439896183644.1904</v>
       </c>
       <c r="T16" s="6">
         <f t="shared" si="1"/>
@@ -1495,43 +1424,43 @@
     </row>
     <row r="17" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="13">
+        <v>60</v>
+      </c>
+      <c r="B17" s="13" t="e">
         <f t="shared" ref="B17:AA17" si="2">B10/B4</f>
-        <v>8.5710151807112139E-2</v>
-      </c>
-      <c r="C17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>2.8911731714418708E-2</v>
-      </c>
-      <c r="D17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>0.1838817854089502</v>
-      </c>
-      <c r="E17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>0.13360488570361934</v>
-      </c>
-      <c r="F17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>9.4765884268007625E-2</v>
-      </c>
-      <c r="G17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>3.6631528968960041E-2</v>
-      </c>
-      <c r="H17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>0.14574903156107299</v>
-      </c>
-      <c r="I17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>4.30809253025565E-2</v>
-      </c>
-      <c r="J17" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J17" s="13" t="e">
         <f t="shared" si="2"/>
-        <v>1.2258464726346834E-2</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K17" s="13" t="e">
         <f t="shared" si="2"/>
@@ -1553,21 +1482,21 @@
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P17" s="13" t="e">
+      <c r="P17" s="13">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q17" s="13" t="e">
+        <v>2.0270759422696519E-2</v>
+      </c>
+      <c r="Q17" s="13">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R17" s="13" t="e">
+        <v>2.1019445677334214E-2</v>
+      </c>
+      <c r="R17" s="13">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S17" s="13" t="e">
+        <v>1.9911840995495259E-2</v>
+      </c>
+      <c r="S17" s="13">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>1.3604246348802499E-2</v>
       </c>
       <c r="T17" s="13" t="e">
         <f t="shared" si="2"/>
@@ -1604,43 +1533,43 @@
     </row>
     <row r="18" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="13">
+        <v>61</v>
+      </c>
+      <c r="B18" s="13" t="e">
         <f t="shared" ref="B18:AA18" si="3">B10/B9</f>
-        <v>0.14726472254348238</v>
-      </c>
-      <c r="C18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>4.7501320636154316E-2</v>
-      </c>
-      <c r="D18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>0.3036070104814495</v>
-      </c>
-      <c r="E18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>0.23194052771069137</v>
-      </c>
-      <c r="F18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>0.16969877481540577</v>
-      </c>
-      <c r="G18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>6.5082843326450909E-2</v>
-      </c>
-      <c r="H18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>0.26252664854667546</v>
-      </c>
-      <c r="I18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>0.10457683216254096</v>
-      </c>
-      <c r="J18" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J18" s="13" t="e">
         <f t="shared" si="3"/>
-        <v>3.0646187164034316E-2</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K18" s="13" t="e">
         <f t="shared" si="3"/>
@@ -1662,21 +1591,21 @@
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P18" s="13" t="e">
+      <c r="P18" s="13">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q18" s="13" t="e">
+        <v>5.8710481860360965E-2</v>
+      </c>
+      <c r="Q18" s="13">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R18" s="13" t="e">
+        <v>6.1286161649409011E-2</v>
+      </c>
+      <c r="R18" s="13">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S18" s="13" t="e">
+        <v>5.7286785664112341E-2</v>
+      </c>
+      <c r="S18" s="13">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>3.9009330557936359E-2</v>
       </c>
       <c r="T18" s="13" t="e">
         <f t="shared" si="3"/>
@@ -1713,43 +1642,43 @@
     </row>
     <row r="19" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B19" s="14">
+        <v>62</v>
+      </c>
+      <c r="B19" s="14" t="e">
         <f t="shared" ref="B19:AA19" si="4">B14/B15</f>
-        <v>1.9463989988422434</v>
-      </c>
-      <c r="C19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>1.5969023152531543</v>
-      </c>
-      <c r="D19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.1311951546146286</v>
-      </c>
-      <c r="E19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.5889544013334715</v>
-      </c>
-      <c r="F19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.4660378507620599</v>
-      </c>
-      <c r="G19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.2323631626940821</v>
-      </c>
-      <c r="H19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.4083499341573376</v>
-      </c>
-      <c r="I19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>3.0062368930240653</v>
-      </c>
-      <c r="J19" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J19" s="14" t="e">
         <f t="shared" si="4"/>
-        <v>2.8914509410747518</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K19" s="14" t="e">
         <f t="shared" si="4"/>
@@ -1771,21 +1700,21 @@
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P19" s="14" t="e">
+      <c r="P19" s="14">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q19" s="14" t="e">
+        <v>2.9826299102526761</v>
+      </c>
+      <c r="Q19" s="14">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R19" s="14" t="e">
+        <v>3.8082100922802176</v>
+      </c>
+      <c r="R19" s="14">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S19" s="14" t="e">
+        <v>4.1272504913265946</v>
+      </c>
+      <c r="S19" s="14">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>2.5150940857263482</v>
       </c>
       <c r="T19" s="14" t="e">
         <f t="shared" si="4"/>
@@ -1822,43 +1751,43 @@
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="14">
+        <v>63</v>
+      </c>
+      <c r="B20" s="14" t="e">
         <f t="shared" ref="B20:AA20" si="5">B14/B21</f>
-        <v>13.217007883660232</v>
-      </c>
-      <c r="C20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>33.61806143212187</v>
-      </c>
-      <c r="D20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>7.0195847956048594</v>
-      </c>
-      <c r="E20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>11.162147585361957</v>
-      </c>
-      <c r="F20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>14.531854183653101</v>
-      </c>
-      <c r="G20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>34.300332447012309</v>
-      </c>
-      <c r="H20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>9.1737351140912811</v>
-      </c>
-      <c r="I20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>28.7466815628107</v>
-      </c>
-      <c r="J20" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J20" s="14" t="e">
         <f t="shared" si="5"/>
-        <v>94.349451225309167</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K20" s="14" t="e">
         <f t="shared" si="5"/>
@@ -1880,21 +1809,21 @@
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P20" s="14" t="e">
+      <c r="P20" s="14">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q20" s="14" t="e">
+        <v>50.802340838330466</v>
+      </c>
+      <c r="Q20" s="14">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R20" s="14" t="e">
+        <v>62.138172628028187</v>
+      </c>
+      <c r="R20" s="14">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S20" s="14" t="e">
+        <v>72.045419261708318</v>
+      </c>
+      <c r="S20" s="14">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>64.47416681480729</v>
       </c>
       <c r="T20" s="14" t="e">
         <f t="shared" si="5"/>
@@ -1931,43 +1860,43 @@
     </row>
     <row r="21" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="6">
+        <v>64</v>
+      </c>
+      <c r="B21" s="6" t="e">
         <f t="shared" ref="B21:AA21" si="6">B10/B13</f>
-        <v>41.99134969769738</v>
-      </c>
-      <c r="C21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>14.040071910541714</v>
-      </c>
-      <c r="D21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>85.475140976383003</v>
-      </c>
-      <c r="E21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>64.055773723835287</v>
-      </c>
-      <c r="F21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>43.353036167173194</v>
-      </c>
-      <c r="G21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>16.90945709916932</v>
-      </c>
-      <c r="H21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>63.769009321122965</v>
-      </c>
-      <c r="I21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>18.089044429834953</v>
-      </c>
-      <c r="J21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J21" s="6" t="e">
         <f t="shared" si="6"/>
-        <v>4.896689848218946</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K21" s="6" t="e">
         <f t="shared" si="6"/>
@@ -1989,21 +1918,21 @@
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P21" s="6" t="e">
+      <c r="P21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q21" s="6" t="e">
+        <v>9.212173932876988</v>
+      </c>
+      <c r="Q21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R21" s="6" t="e">
+        <v>9.3340369610158742</v>
+      </c>
+      <c r="R21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S21" s="6" t="e">
+        <v>8.4668811182033217</v>
+      </c>
+      <c r="S21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>5.4595509704075598</v>
       </c>
       <c r="T21" s="6" t="e">
         <f t="shared" si="6"/>
@@ -2040,43 +1969,43 @@
     </row>
     <row r="22" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="13">
+        <v>65</v>
+      </c>
+      <c r="B22" s="13" t="e">
         <f t="shared" ref="B22:AA22" si="7">B7/B9</f>
-        <v>0.71815825587811088</v>
-      </c>
-      <c r="C22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.64296548999008429</v>
-      </c>
-      <c r="D22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.65108679771641964</v>
-      </c>
-      <c r="E22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.73600488588855351</v>
-      </c>
-      <c r="F22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.79070192487031521</v>
-      </c>
-      <c r="G22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.77667624522899548</v>
-      </c>
-      <c r="H22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>0.80121049011285517</v>
-      </c>
-      <c r="I22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>1.4274358619762304</v>
-      </c>
-      <c r="J22" s="13">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J22" s="13" t="e">
         <f t="shared" si="7"/>
-        <v>1.4999866971338565</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="K22" s="13" t="e">
         <f t="shared" si="7"/>
@@ -2098,21 +2027,21 @@
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="P22" s="13" t="e">
+      <c r="P22" s="13">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q22" s="13" t="e">
+        <v>1.8966467016698216</v>
+      </c>
+      <c r="Q22" s="13">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R22" s="13" t="e">
+        <v>1.9162738933050549</v>
+      </c>
+      <c r="R22" s="13">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S22" s="13" t="e">
+        <v>1.8776975518939529</v>
+      </c>
+      <c r="S22" s="13">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>1.8677545561822233</v>
       </c>
       <c r="T22" s="13" t="e">
         <f t="shared" si="7"/>
@@ -3132,6 +3061,62 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB258A72-9464-5845-A57C-12441F1547AB}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="18">
+        <v>6.7299999999999999E-2</v>
+      </c>
+      <c r="B2">
+        <f>1000/A2</f>
+        <v>14858.841010401189</v>
+      </c>
+      <c r="C2" s="19">
+        <v>247029168</v>
+      </c>
+      <c r="D2" s="16">
+        <f>B2*C2</f>
+        <v>3670567132243.6851</v>
+      </c>
+      <c r="F2" s="16">
+        <v>939896509146.34131</v>
+      </c>
+      <c r="G2" s="16">
+        <v>282009237804.87799</v>
+      </c>
+      <c r="H2" s="17">
+        <f>F2+G2</f>
+        <v>1221905746951.2192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3163,125 +3148,125 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1">
         <v>3734</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C3" s="1">
         <v>6365</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="C4" s="3">
         <v>6267</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="C5" s="3">
         <v>5029</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3">
         <v>10794</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3">
         <v>3356</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="3">
         <v>16348</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="C9" s="3">
         <v>1528</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" s="3">
         <v>11009</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: adjust the prompt for the gemini 3.5-flash-lite and some improvement on field understanding
</commit_message>
<xml_diff>
--- a/data/ground_truth/ARCI.xlsx
+++ b/data/ground_truth/ARCI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadnajmirahmani/Belajar/ProjectDatasaur/data/ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A02C08A-CDC6-E84B-9040-C2905D8A04C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C195CF6-CF38-F34A-924F-C494CEC95355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29300" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
   <si>
     <t>Perusahaan</t>
   </si>
@@ -251,6 +273,9 @@
   </si>
   <si>
     <t>Converted</t>
+  </si>
+  <si>
+    <t>25235000000.0</t>
   </si>
 </sst>
 </file>
@@ -263,7 +288,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -274,11 +299,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Tahoma"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -303,6 +330,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -332,7 +365,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -344,12 +377,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -368,6 +396,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
@@ -597,9 +626,9 @@
     <col min="10" max="10" width="17.5" customWidth="1"/>
     <col min="11" max="11" width="17.1640625" customWidth="1"/>
     <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="8.6640625" customWidth="1"/>
-    <col min="16" max="16" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="8.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" bestFit="1" customWidth="1"/>
@@ -612,7 +641,7 @@
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>66</v>
       </c>
       <c r="E1" s="2"/>
@@ -753,24 +782,52 @@
       <c r="A4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8">
+      <c r="B4" s="5">
+        <v>19189496535714</v>
+      </c>
+      <c r="C4" s="5">
+        <v>18047481428571</v>
+      </c>
+      <c r="D4" s="5">
+        <v>17227573439597</v>
+      </c>
+      <c r="E4" s="5">
+        <v>15886383333333</v>
+      </c>
+      <c r="F4" s="5">
+        <v>14580815081169</v>
+      </c>
+      <c r="G4" s="5">
+        <v>14619914494196</v>
+      </c>
+      <c r="H4" s="5">
+        <v>13980610613893</v>
+      </c>
+      <c r="I4" s="5">
+        <v>12766261376702</v>
+      </c>
+      <c r="J4" s="5">
+        <v>13503189704433</v>
+      </c>
+      <c r="K4" s="5">
+        <v>12882307892235</v>
+      </c>
+      <c r="L4" s="5">
+        <v>12381820970724</v>
+      </c>
+      <c r="M4" s="5">
+        <v>12334644565217</v>
+      </c>
+      <c r="N4" s="5">
+        <v>11325048408408</v>
+      </c>
+      <c r="O4" s="5">
+        <v>11020926611446</v>
+      </c>
+      <c r="P4" s="5">
         <v>11286421729559.748</v>
       </c>
-      <c r="Q4" s="16">
+      <c r="Q4" s="5">
         <v>11028397774390.242</v>
       </c>
       <c r="R4" s="5">
@@ -780,33 +837,61 @@
         <v>9966590200860.832</v>
       </c>
       <c r="T4" s="5"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-      <c r="AA4" s="9"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="7"/>
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6">
+      <c r="B5" s="5">
+        <v>2979297232143</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2927146258503</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2887927147651</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2184739283333</v>
+      </c>
+      <c r="F5" s="5">
+        <v>1349429951299</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1366961492537</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1499000096931</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1229991785174</v>
+      </c>
+      <c r="J5" s="5">
+        <v>1289915648604</v>
+      </c>
+      <c r="K5" s="5">
+        <v>1417295277338</v>
+      </c>
+      <c r="L5" s="5">
+        <v>1457045855162</v>
+      </c>
+      <c r="M5" s="5">
+        <v>1741458509317</v>
+      </c>
+      <c r="N5" s="5">
+        <v>973281951952</v>
+      </c>
+      <c r="O5" s="5">
+        <v>1191006762048</v>
+      </c>
+      <c r="P5" s="5">
         <v>1370668490566.0376</v>
       </c>
       <c r="Q5" s="5">
@@ -819,111 +904,195 @@
         <v>1052012410329.9857</v>
       </c>
       <c r="T5" s="5"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
-      <c r="AA5" s="9"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="7"/>
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8">
+      <c r="B6" s="5">
+        <v>409296625000</v>
+      </c>
+      <c r="C6" s="5">
+        <v>671137295918</v>
+      </c>
+      <c r="D6" s="5">
+        <v>417496359060</v>
+      </c>
+      <c r="E6" s="5">
+        <v>390399600000</v>
+      </c>
+      <c r="F6" s="5">
+        <v>70624772727</v>
+      </c>
+      <c r="G6" s="5">
+        <v>47900281924</v>
+      </c>
+      <c r="H6" s="5">
+        <v>73296995153</v>
+      </c>
+      <c r="I6" s="5">
+        <v>142554009077</v>
+      </c>
+      <c r="J6" s="5">
+        <v>175804548440</v>
+      </c>
+      <c r="K6" s="5">
+        <v>54720950872</v>
+      </c>
+      <c r="L6" s="5">
+        <v>143608274268</v>
+      </c>
+      <c r="M6" s="5">
+        <v>277259378882</v>
+      </c>
+      <c r="N6" s="5">
+        <v>56026486486</v>
+      </c>
+      <c r="O6" s="5">
+        <v>95256641566</v>
+      </c>
+      <c r="P6" s="5">
         <v>162569716981.13208</v>
       </c>
       <c r="Q6" s="5">
         <v>146141859756.09753</v>
       </c>
-      <c r="R6" s="20">
+      <c r="R6" s="17">
         <v>184978038633</v>
       </c>
       <c r="S6" s="5">
         <v>331786255380.20087</v>
       </c>
       <c r="T6" s="5"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
-      <c r="AA6" s="9"/>
+      <c r="U6" s="7"/>
+      <c r="V6" s="7"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="7"/>
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8">
+      <c r="B7" s="5">
+        <v>11803092071429</v>
+      </c>
+      <c r="C7" s="5">
+        <v>11364988384354</v>
+      </c>
+      <c r="D7" s="5">
+        <v>11138182298658</v>
+      </c>
+      <c r="E7" s="5">
+        <v>10153818500000</v>
+      </c>
+      <c r="F7" s="5">
+        <v>9575570211039</v>
+      </c>
+      <c r="G7" s="5">
+        <v>9921723548922</v>
+      </c>
+      <c r="H7" s="5">
+        <v>9570979579968</v>
+      </c>
+      <c r="I7" s="5">
+        <v>8849227080182</v>
+      </c>
+      <c r="J7" s="5">
+        <v>9266104597701</v>
+      </c>
+      <c r="K7" s="5">
+        <v>8790164072900</v>
+      </c>
+      <c r="L7" s="5">
+        <v>8335133990755</v>
+      </c>
+      <c r="M7" s="5">
+        <v>8302537375776</v>
+      </c>
+      <c r="N7" s="5">
+        <v>7478349204204</v>
+      </c>
+      <c r="O7" s="5">
+        <v>7212862966867</v>
+      </c>
+      <c r="P7" s="5">
         <v>7390895959119</v>
       </c>
       <c r="Q7" s="5">
         <v>7248177850609.7549</v>
       </c>
-      <c r="R7" s="16">
+      <c r="R7" s="13">
         <v>6892214918276.375</v>
       </c>
       <c r="S7" s="5">
         <v>6491908593974.1758</v>
       </c>
       <c r="T7" s="5"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-      <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
-      <c r="AA7" s="9"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="7"/>
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8">
+      <c r="B8" s="5">
+        <v>1090018553571</v>
+      </c>
+      <c r="C8" s="5">
+        <v>834453248299</v>
+      </c>
+      <c r="D8" s="5">
+        <v>956825738255</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1852997600000</v>
+      </c>
+      <c r="F8" s="5">
+        <v>1556383457792</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1315414726368</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1033713780291</v>
+      </c>
+      <c r="I8" s="5">
+        <v>789302329803</v>
+      </c>
+      <c r="J8" s="5">
+        <v>819519967159</v>
+      </c>
+      <c r="K8" s="5">
+        <v>767365721078</v>
+      </c>
+      <c r="L8" s="5">
+        <v>757654699538</v>
+      </c>
+      <c r="M8" s="5">
+        <v>759932531056</v>
+      </c>
+      <c r="N8" s="5">
+        <v>1956975885886</v>
+      </c>
+      <c r="O8" s="5">
+        <v>1691064608434</v>
+      </c>
+      <c r="P8" s="5">
         <v>1503778443396</v>
       </c>
       <c r="Q8" s="5">
@@ -936,72 +1105,128 @@
         <v>1468543529411.7646</v>
       </c>
       <c r="T8" s="5"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8">
+      <c r="B9" s="5">
+        <v>7353328160714</v>
+      </c>
+      <c r="C9" s="5">
+        <v>6663430374150</v>
+      </c>
+      <c r="D9" s="5">
+        <v>6077018808725</v>
+      </c>
+      <c r="E9" s="5">
+        <v>5721647966667</v>
+      </c>
+      <c r="F9" s="5">
+        <v>4997574155844</v>
+      </c>
+      <c r="G9" s="5">
+        <v>4693880281924</v>
+      </c>
+      <c r="H9" s="5">
+        <v>4408820920840</v>
+      </c>
+      <c r="I9" s="5">
+        <v>3915716959153</v>
+      </c>
+      <c r="J9" s="5">
+        <v>4236824334975</v>
+      </c>
+      <c r="K9" s="5">
+        <v>4090532551506</v>
+      </c>
+      <c r="L9" s="5">
+        <v>4045221879815</v>
+      </c>
+      <c r="M9" s="5">
+        <v>4028813990683</v>
+      </c>
+      <c r="N9" s="5">
+        <v>3842490600601</v>
+      </c>
+      <c r="O9" s="5">
+        <v>3811828644578</v>
+      </c>
+      <c r="P9" s="5">
         <v>3896822720126</v>
       </c>
       <c r="Q9" s="5">
         <v>3782433124999.9995</v>
       </c>
-      <c r="R9" s="16">
+      <c r="R9" s="13">
         <v>3670567132243.6851</v>
       </c>
       <c r="S9" s="5">
         <v>3475782496413.1997</v>
       </c>
       <c r="T9" s="5"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
-      <c r="AA9" s="9"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="7"/>
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8">
+      <c r="B10" s="5">
+        <v>1433061178571</v>
+      </c>
+      <c r="C10" s="5">
+        <v>506688826531</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1708406359060</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1174628250000</v>
+      </c>
+      <c r="F10" s="5">
+        <v>566102840909</v>
+      </c>
+      <c r="G10" s="5">
+        <v>170563117745</v>
+      </c>
+      <c r="H10" s="5">
+        <v>168944313409</v>
+      </c>
+      <c r="I10" s="5">
+        <v>-58920756430</v>
+      </c>
+      <c r="J10" s="5">
+        <v>-63835024631</v>
+      </c>
+      <c r="K10" s="5">
+        <v>-66303692552</v>
+      </c>
+      <c r="L10" s="5">
+        <v>224495208012</v>
+      </c>
+      <c r="M10" s="5">
+        <v>169652484472</v>
+      </c>
+      <c r="N10" s="5">
+        <v>109699054054</v>
+      </c>
+      <c r="O10" s="5">
+        <v>73026460843</v>
+      </c>
+      <c r="P10" s="5">
         <v>228784339623</v>
       </c>
       <c r="Q10" s="5">
@@ -1014,32 +1239,60 @@
         <v>135587948350.07175</v>
       </c>
       <c r="T10" s="5"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="9"/>
-      <c r="AA10" s="9"/>
+      <c r="U10" s="7"/>
+      <c r="V10" s="7"/>
+      <c r="W10" s="7"/>
+      <c r="X10" s="7"/>
+      <c r="Y10" s="7"/>
+      <c r="Z10" s="7"/>
+      <c r="AA10" s="7"/>
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
+      <c r="B11" s="5">
+        <v>5755149375000</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2328361428571</v>
+      </c>
+      <c r="D11" s="5">
+        <v>8326003741611</v>
+      </c>
+      <c r="E11" s="5">
+        <v>5478341016667</v>
+      </c>
+      <c r="F11" s="5">
+        <v>3125823311688</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1505426948590</v>
+      </c>
+      <c r="H11" s="5">
+        <v>4646508513732</v>
+      </c>
+      <c r="I11" s="5">
+        <v>3257286263238</v>
+      </c>
+      <c r="J11" s="5">
+        <v>2345676732348</v>
+      </c>
+      <c r="K11" s="5">
+        <v>903510570523</v>
+      </c>
+      <c r="L11" s="5">
+        <v>3846390878274</v>
+      </c>
+      <c r="M11" s="5">
+        <v>2675790916149</v>
+      </c>
+      <c r="N11" s="5">
+        <v>1732177147147</v>
+      </c>
+      <c r="O11" s="5">
+        <v>851079141566</v>
+      </c>
       <c r="P11" s="5">
         <v>3403714968553</v>
       </c>
@@ -1053,33 +1306,61 @@
         <v>1149631348637.0159</v>
       </c>
       <c r="T11" s="5"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
-      <c r="AA11" s="9"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7"/>
+      <c r="AA11" s="7"/>
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8">
+      <c r="B12" s="5">
+        <v>1645245910714</v>
+      </c>
+      <c r="C12" s="5">
+        <v>827912023810</v>
+      </c>
+      <c r="D12" s="5">
+        <v>879448909396</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1450888483333</v>
+      </c>
+      <c r="F12" s="5">
+        <v>675487191558</v>
+      </c>
+      <c r="G12" s="5">
+        <v>355914096186</v>
+      </c>
+      <c r="H12" s="5">
+        <v>1454744103393</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1002810680787</v>
+      </c>
+      <c r="J12" s="5">
+        <v>776953957307</v>
+      </c>
+      <c r="K12" s="5">
+        <v>332297448494</v>
+      </c>
+      <c r="L12" s="5">
+        <v>327001402157</v>
+      </c>
+      <c r="M12" s="5">
+        <v>9790403727</v>
+      </c>
+      <c r="N12" s="5">
+        <v>905774459459</v>
+      </c>
+      <c r="O12" s="5">
+        <v>375205030120</v>
+      </c>
+      <c r="P12" s="5">
         <v>853635345912</v>
       </c>
       <c r="Q12" s="5">
@@ -1092,32 +1373,60 @@
         <v>522079942611.19086</v>
       </c>
       <c r="T12" s="5"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
-      <c r="AA12" s="9"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="7"/>
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
+      <c r="B13" s="5">
+        <v>25235000000</v>
+      </c>
+      <c r="C13" s="5">
+        <v>25235000000</v>
+      </c>
+      <c r="D13" s="5">
+        <v>25235000000</v>
+      </c>
+      <c r="E13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="F13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="G13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="H13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="I13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="J13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="K13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="L13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="M13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="N13" s="5">
+        <v>24835000000</v>
+      </c>
+      <c r="O13" s="5">
+        <v>24835000000</v>
+      </c>
       <c r="P13" s="5">
         <v>24835000000</v>
       </c>
@@ -1131,13 +1440,13 @@
         <v>24835000000</v>
       </c>
       <c r="T13" s="5"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
-      <c r="AA13" s="9"/>
+      <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
+      <c r="X13" s="7"/>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="7"/>
+      <c r="AA13" s="7"/>
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
@@ -1152,27 +1461,13 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="5">
-        <v>444</v>
-      </c>
-      <c r="L14" s="5">
-        <v>448</v>
-      </c>
-      <c r="M14" s="5">
-        <v>454</v>
-      </c>
-      <c r="N14" s="5">
-        <v>458</v>
-      </c>
-      <c r="O14" s="5">
-        <v>454</v>
-      </c>
-      <c r="P14" s="5">
-        <v>468</v>
-      </c>
-      <c r="Q14" s="5">
-        <v>580</v>
-      </c>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
       <c r="R14" s="5">
         <v>610</v>
       </c>
@@ -1182,87 +1477,87 @@
       <c r="T14" s="5">
         <v>725</v>
       </c>
-      <c r="U14" s="9">
+      <c r="U14" s="7">
         <v>570</v>
       </c>
-      <c r="V14" s="9">
+      <c r="V14" s="7">
         <v>570</v>
       </c>
       <c r="W14" s="4">
         <v>570</v>
       </c>
-      <c r="X14" s="9">
+      <c r="X14" s="7">
         <v>570</v>
       </c>
-      <c r="Y14" s="9">
+      <c r="Y14" s="7">
         <v>570</v>
       </c>
-      <c r="Z14" s="9">
+      <c r="Z14" s="7">
         <v>1140</v>
       </c>
-      <c r="AA14" s="9">
+      <c r="AA14" s="7">
         <v>1140</v>
       </c>
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="6" t="e">
+      <c r="B15" s="6">
         <f t="shared" ref="B15:AA15" si="0">B9/B13</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C15" s="6" t="e">
+        <v>291.3940226159699</v>
+      </c>
+      <c r="C15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D15" s="6" t="e">
+        <v>264.05509705369525</v>
+      </c>
+      <c r="D15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E15" s="6" t="e">
+        <v>240.81707187339012</v>
+      </c>
+      <c r="E15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F15" s="6" t="e">
+        <v>230.38646936448561</v>
+      </c>
+      <c r="F15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G15" s="6" t="e">
+        <v>201.23109143724582</v>
+      </c>
+      <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H15" s="6" t="e">
+        <v>189.00262862589088</v>
+      </c>
+      <c r="H15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I15" s="6" t="e">
+        <v>177.52449852385746</v>
+      </c>
+      <c r="I15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J15" s="6" t="e">
+        <v>157.66929571785786</v>
+      </c>
+      <c r="J15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K15" s="6" t="e">
+        <v>170.59892631266359</v>
+      </c>
+      <c r="K15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L15" s="6" t="e">
+        <v>164.70837735075497</v>
+      </c>
+      <c r="L15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M15" s="6" t="e">
+        <v>162.88390899194684</v>
+      </c>
+      <c r="M15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N15" s="6" t="e">
+        <v>162.22323296488827</v>
+      </c>
+      <c r="N15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O15" s="6" t="e">
+        <v>154.72078117982684</v>
+      </c>
+      <c r="O15" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>153.48615440217435</v>
       </c>
       <c r="P15" s="6">
         <f t="shared" si="0"/>
@@ -1296,82 +1591,82 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X15" s="12" t="e">
+      <c r="X15" s="9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y15" s="12" t="e">
+      <c r="Y15" s="9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z15" s="12" t="e">
+      <c r="Z15" s="9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA15" s="12" t="e">
+      <c r="AA15" s="9" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B16" s="6">
         <f t="shared" ref="B16:AA16" si="1">B5-B7</f>
-        <v>0</v>
+        <v>-8823794839286</v>
       </c>
       <c r="C16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8437842125851</v>
       </c>
       <c r="D16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8250255151007</v>
       </c>
       <c r="E16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-7969079216667</v>
       </c>
       <c r="F16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8226140259740</v>
       </c>
       <c r="G16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8554762056385</v>
       </c>
       <c r="H16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8071979483037</v>
       </c>
       <c r="I16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-7619235295008</v>
       </c>
       <c r="J16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-7976188949097</v>
       </c>
       <c r="K16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-7372868795562</v>
       </c>
       <c r="L16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6878088135593</v>
       </c>
       <c r="M16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6561078866459</v>
       </c>
       <c r="N16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6505067252252</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-6021856204819</v>
       </c>
       <c r="P16" s="6">
         <f t="shared" si="1"/>
@@ -1405,518 +1700,518 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="X16" s="12">
+      <c r="X16" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Y16" s="12">
+      <c r="Y16" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Z16" s="12">
+      <c r="Z16" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AA16" s="12">
+      <c r="AA16" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="13" t="e">
+      <c r="B17" s="10">
         <f t="shared" ref="B17:AA17" si="2">B10/B4</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C17" s="13" t="e">
+        <v>7.4679456853070522E-2</v>
+      </c>
+      <c r="C17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D17" s="13" t="e">
+        <v>2.8075320566827679E-2</v>
+      </c>
+      <c r="D17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E17" s="13" t="e">
+        <v>9.916697583963191E-2</v>
+      </c>
+      <c r="E17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F17" s="13" t="e">
+        <v>7.3939311758604048E-2</v>
+      </c>
+      <c r="F17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G17" s="13" t="e">
+        <v>3.8825184858157696E-2</v>
+      </c>
+      <c r="G17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H17" s="13" t="e">
+        <v>1.1666492154431704E-2</v>
+      </c>
+      <c r="H17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I17" s="13" t="e">
+        <v>1.2084187026932456E-2</v>
+      </c>
+      <c r="I17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J17" s="13" t="e">
+        <v>-4.6153493721762901E-3</v>
+      </c>
+      <c r="J17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K17" s="13" t="e">
+        <v>-4.7274033786286378E-3</v>
+      </c>
+      <c r="K17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L17" s="13" t="e">
+        <v>-5.1468799773032531E-3</v>
+      </c>
+      <c r="L17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M17" s="13" t="e">
+        <v>1.8131033273926681E-2</v>
+      </c>
+      <c r="M17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N17" s="13" t="e">
+        <v>1.3754144562090618E-2</v>
+      </c>
+      <c r="N17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O17" s="13" t="e">
+        <v>9.6864092847988772E-3</v>
+      </c>
+      <c r="O17" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P17" s="13">
+        <v>6.6261634268716509E-3</v>
+      </c>
+      <c r="P17" s="10">
         <f t="shared" si="2"/>
         <v>2.0270759422696519E-2</v>
       </c>
-      <c r="Q17" s="13">
+      <c r="Q17" s="10">
         <f t="shared" si="2"/>
         <v>2.1019445677334214E-2</v>
       </c>
-      <c r="R17" s="13">
+      <c r="R17" s="10">
         <f t="shared" si="2"/>
         <v>1.9911840995495259E-2</v>
       </c>
-      <c r="S17" s="13">
+      <c r="S17" s="10">
         <f t="shared" si="2"/>
         <v>1.3604246348802499E-2</v>
       </c>
-      <c r="T17" s="13" t="e">
+      <c r="T17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="U17" s="13" t="e">
+      <c r="U17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V17" s="13" t="e">
+      <c r="V17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W17" s="13" t="e">
+      <c r="W17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X17" s="13" t="e">
+      <c r="X17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y17" s="13" t="e">
+      <c r="Y17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z17" s="13" t="e">
+      <c r="Z17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA17" s="13" t="e">
+      <c r="AA17" s="10" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="13" t="e">
+      <c r="B18" s="10">
         <f t="shared" ref="B18:AA18" si="3">B10/B9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C18" s="13" t="e">
+        <v>0.19488606345998455</v>
+      </c>
+      <c r="C18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D18" s="13" t="e">
+        <v>7.604023724726533E-2</v>
+      </c>
+      <c r="D18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E18" s="13" t="e">
+        <v>0.2811257316839596</v>
+      </c>
+      <c r="E18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F18" s="13" t="e">
+        <v>0.20529544229968585</v>
+      </c>
+      <c r="F18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G18" s="13" t="e">
+        <v>0.11327552593632209</v>
+      </c>
+      <c r="G18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H18" s="13" t="e">
+        <v>3.6337338726305769E-2</v>
+      </c>
+      <c r="H18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I18" s="13" t="e">
+        <v>3.8319613439144071E-2</v>
+      </c>
+      <c r="I18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J18" s="13" t="e">
+        <v>-1.504724602023968E-2</v>
+      </c>
+      <c r="J18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K18" s="13" t="e">
+        <v>-1.5066714969521309E-2</v>
+      </c>
+      <c r="K18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L18" s="13" t="e">
+        <v>-1.6209061220546737E-2</v>
+      </c>
+      <c r="L18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M18" s="13" t="e">
+        <v>5.5496389241884263E-2</v>
+      </c>
+      <c r="M18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N18" s="13" t="e">
+        <v>4.2109783391424092E-2</v>
+      </c>
+      <c r="N18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O18" s="13" t="e">
+        <v>2.85489453212565E-2</v>
+      </c>
+      <c r="O18" s="10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P18" s="13">
+        <v>1.9157855101087477E-2</v>
+      </c>
+      <c r="P18" s="10">
         <f t="shared" si="3"/>
         <v>5.8710481860360965E-2</v>
       </c>
-      <c r="Q18" s="13">
+      <c r="Q18" s="10">
         <f t="shared" si="3"/>
         <v>6.1286161649409011E-2</v>
       </c>
-      <c r="R18" s="13">
+      <c r="R18" s="10">
         <f t="shared" si="3"/>
         <v>5.7286785664112341E-2</v>
       </c>
-      <c r="S18" s="13">
+      <c r="S18" s="10">
         <f t="shared" si="3"/>
         <v>3.9009330557936359E-2</v>
       </c>
-      <c r="T18" s="13" t="e">
+      <c r="T18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="U18" s="13" t="e">
+      <c r="U18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V18" s="13" t="e">
+      <c r="V18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W18" s="13" t="e">
+      <c r="W18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X18" s="13" t="e">
+      <c r="X18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y18" s="13" t="e">
+      <c r="Y18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z18" s="13" t="e">
+      <c r="Z18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA18" s="13" t="e">
+      <c r="AA18" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="14" t="e">
+      <c r="B19" s="11">
         <f t="shared" ref="B19:AA19" si="4">B14/B15</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="C19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="D19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="E19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="G19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="H19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="I19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="J19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="K19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="L19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="M19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="N19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O19" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="O19" s="11">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P19" s="14">
+        <v>0</v>
+      </c>
+      <c r="P19" s="11">
         <f t="shared" si="4"/>
-        <v>2.9826299102526761</v>
-      </c>
-      <c r="Q19" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="11">
         <f t="shared" si="4"/>
-        <v>3.8082100922802176</v>
-      </c>
-      <c r="R19" s="14">
+        <v>0</v>
+      </c>
+      <c r="R19" s="11">
         <f t="shared" si="4"/>
         <v>4.1272504913265946</v>
       </c>
-      <c r="S19" s="14">
+      <c r="S19" s="11">
         <f t="shared" si="4"/>
         <v>2.5150940857263482</v>
       </c>
-      <c r="T19" s="14" t="e">
+      <c r="T19" s="11" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="U19" s="14" t="e">
+      <c r="U19" s="11" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V19" s="14" t="e">
+      <c r="V19" s="11" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W19" s="14" t="e">
+      <c r="W19" s="11" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X19" s="12" t="e">
+      <c r="X19" s="9" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y19" s="12" t="e">
+      <c r="Y19" s="9" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z19" s="12" t="e">
+      <c r="Z19" s="9" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA19" s="12" t="e">
+      <c r="AA19" s="9" t="e">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="14" t="e">
+      <c r="B20" s="11">
         <f t="shared" ref="B20:AA20" si="5">B14/B21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="C20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="D20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="E20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="F20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="G20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="H20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="I20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="J20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="K20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="L20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="M20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="N20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O20" s="14" t="e">
+        <v>0</v>
+      </c>
+      <c r="O20" s="11">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P20" s="14">
+        <v>0</v>
+      </c>
+      <c r="P20" s="11">
         <f t="shared" si="5"/>
-        <v>50.802340838330466</v>
-      </c>
-      <c r="Q20" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="11">
         <f t="shared" si="5"/>
-        <v>62.138172628028187</v>
-      </c>
-      <c r="R20" s="14">
+        <v>0</v>
+      </c>
+      <c r="R20" s="11">
         <f t="shared" si="5"/>
         <v>72.045419261708318</v>
       </c>
-      <c r="S20" s="14">
+      <c r="S20" s="11">
         <f t="shared" si="5"/>
         <v>64.47416681480729</v>
       </c>
-      <c r="T20" s="14" t="e">
+      <c r="T20" s="11" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="U20" s="14" t="e">
+      <c r="U20" s="11" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V20" s="14" t="e">
+      <c r="V20" s="11" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W20" s="14" t="e">
+      <c r="W20" s="11" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X20" s="12" t="e">
+      <c r="X20" s="9" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y20" s="12" t="e">
+      <c r="Y20" s="9" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z20" s="12" t="e">
+      <c r="Z20" s="9" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA20" s="12" t="e">
+      <c r="AA20" s="9" t="e">
         <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="21" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="6" t="e">
+      <c r="B21" s="6">
         <f t="shared" ref="B21:AA21" si="6">B10/B13</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C21" s="6" t="e">
+        <v>56.788633983396075</v>
+      </c>
+      <c r="C21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D21" s="6" t="e">
+        <v>20.07881222631266</v>
+      </c>
+      <c r="D21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E21" s="6" t="e">
+        <v>67.699875532395481</v>
+      </c>
+      <c r="E21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F21" s="6" t="e">
+        <v>47.2972921280451</v>
+      </c>
+      <c r="F21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G21" s="6" t="e">
+        <v>22.79455771729414</v>
+      </c>
+      <c r="G21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" s="6" t="e">
+        <v>6.8678525365411716</v>
+      </c>
+      <c r="H21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I21" s="6" t="e">
+        <v>6.8026701594121199</v>
+      </c>
+      <c r="I21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J21" s="6" t="e">
+        <v>-2.3724886825045299</v>
+      </c>
+      <c r="J21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K21" s="6" t="e">
+        <v>-2.570365396859271</v>
+      </c>
+      <c r="K21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L21" s="6" t="e">
+        <v>-2.669768172015301</v>
+      </c>
+      <c r="L21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M21" s="6" t="e">
+        <v>9.0394688146567344</v>
+      </c>
+      <c r="M21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N21" s="6" t="e">
+        <v>6.8311852012079726</v>
+      </c>
+      <c r="N21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O21" s="6" t="e">
+        <v>4.4171151219649687</v>
+      </c>
+      <c r="O21" s="6">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>2.9404655060599958</v>
       </c>
       <c r="P21" s="6">
         <f t="shared" si="6"/>
@@ -1950,158 +2245,230 @@
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X21" s="12" t="e">
+      <c r="X21" s="9" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y21" s="12" t="e">
+      <c r="Y21" s="9" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z21" s="12" t="e">
+      <c r="Z21" s="9" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA21" s="12" t="e">
+      <c r="AA21" s="9" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="22" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="13" t="e">
+      <c r="B22" s="10">
         <f t="shared" ref="B22:AA22" si="7">B7/B9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C22" s="13" t="e">
+        <v>1.605136043633735</v>
+      </c>
+      <c r="C22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D22" s="13" t="e">
+        <v>1.7055762191863135</v>
+      </c>
+      <c r="D22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E22" s="13" t="e">
+        <v>1.8328365682637844</v>
+      </c>
+      <c r="E22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F22" s="13" t="e">
+        <v>1.7746318122250446</v>
+      </c>
+      <c r="F22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G22" s="13" t="e">
+        <v>1.9160436468644775</v>
+      </c>
+      <c r="G22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H22" s="13" t="e">
+        <v>2.1137572654186081</v>
+      </c>
+      <c r="H22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I22" s="13" t="e">
+        <v>2.1708705687561629</v>
+      </c>
+      <c r="I22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J22" s="13" t="e">
+        <v>2.2599251101377247</v>
+      </c>
+      <c r="J22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K22" s="13" t="e">
+        <v>2.1870400717842546</v>
+      </c>
+      <c r="K22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L22" s="13" t="e">
+        <v>2.1489045649236429</v>
+      </c>
+      <c r="L22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M22" s="13" t="e">
+        <v>2.0604887045494253</v>
+      </c>
+      <c r="M22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N22" s="13" t="e">
+        <v>2.0607894519271368</v>
+      </c>
+      <c r="N22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O22" s="13" t="e">
+        <v>1.9462244626009806</v>
+      </c>
+      <c r="O22" s="10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P22" s="13">
+        <v>1.8922316922946367</v>
+      </c>
+      <c r="P22" s="10">
         <f t="shared" si="7"/>
         <v>1.8966467016698216</v>
       </c>
-      <c r="Q22" s="13">
+      <c r="Q22" s="10">
         <f t="shared" si="7"/>
         <v>1.9162738933050549</v>
       </c>
-      <c r="R22" s="13">
+      <c r="R22" s="10">
         <f t="shared" si="7"/>
         <v>1.8776975518939529</v>
       </c>
-      <c r="S22" s="13">
+      <c r="S22" s="10">
         <f t="shared" si="7"/>
         <v>1.8677545561822233</v>
       </c>
-      <c r="T22" s="13" t="e">
+      <c r="T22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="U22" s="13" t="e">
+      <c r="U22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V22" s="13" t="e">
+      <c r="V22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W22" s="13" t="e">
+      <c r="W22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="X22" s="13" t="e">
+      <c r="X22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y22" s="13" t="e">
+      <c r="Y22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z22" s="13" t="e">
+      <c r="Z22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA22" s="13" t="e">
+      <c r="AA22" s="10" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="18">
+        <v>19189496535714</v>
+      </c>
+      <c r="E25" s="18">
+        <v>2979297232143</v>
+      </c>
+      <c r="F25" s="18">
+        <v>409296625000</v>
+      </c>
+      <c r="G25" s="18">
+        <v>11803092071429</v>
+      </c>
+      <c r="H25" s="18">
+        <v>1090018553571</v>
+      </c>
+      <c r="I25" s="18">
+        <v>7353328160714</v>
+      </c>
+      <c r="J25" s="18">
+        <v>1433061178571</v>
+      </c>
+      <c r="K25" s="18">
+        <v>5755149375000</v>
+      </c>
+      <c r="L25" s="18">
+        <v>1645245910714</v>
+      </c>
+      <c r="M25" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
     <row r="26" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" cm="1">
+        <f t="array" ref="D27:D36">TRANSPOSE(D25:M25)</f>
+        <v>19189496535714</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <v>2979297232143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D29">
+        <v>409296625000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D30">
+        <v>11803092071429</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D31">
+        <v>1090018553571</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>7353328160714</v>
+      </c>
+    </row>
+    <row r="33" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>1433061178571</v>
+      </c>
+    </row>
+    <row r="34" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>5755149375000</v>
+      </c>
+    </row>
+    <row r="35" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>1645245910714</v>
+      </c>
+    </row>
+    <row r="36" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D36" t="str">
+        <v>25235000000.0</v>
+      </c>
+    </row>
+    <row r="37" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3086,27 +3453,27 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="18">
-        <v>6.7299999999999999E-2</v>
+      <c r="A2" s="15">
+        <v>6.0900000000000003E-2</v>
       </c>
       <c r="B2">
         <f>1000/A2</f>
-        <v>14858.841010401189</v>
-      </c>
-      <c r="C2" s="19">
-        <v>247029168</v>
-      </c>
-      <c r="D2" s="16">
+        <v>16420.361247947454</v>
+      </c>
+      <c r="C2" s="16">
+        <v>822344253</v>
+      </c>
+      <c r="D2" s="13">
         <f>B2*C2</f>
-        <v>3670567132243.6851</v>
-      </c>
-      <c r="F2" s="16">
+        <v>13503189704433.496</v>
+      </c>
+      <c r="F2" s="13">
         <v>939896509146.34131</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="13">
         <v>282009237804.87799</v>
       </c>
-      <c r="H2" s="17">
+      <c r="H2" s="14">
         <f>F2+G2</f>
         <v>1221905746951.2192</v>
       </c>

</xml_diff>

<commit_message>
feat: add the share price fetch to get the share price on an exact date
</commit_message>
<xml_diff>
--- a/data/ground_truth/ARCI.xlsx
+++ b/data/ground_truth/ARCI.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadnajmirahmani/Belajar/ProjectDatasaur/data/ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C195CF6-CF38-F34A-924F-C494CEC95355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A571F0D3-469A-BA45-939B-3809BBF92057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29300" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
-    <sheet name="lokasi kebun" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="lokasi kebun" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,44 +30,175 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="c1H/Q4ZdR4yLnEJr0IZqFh3FObkfqorOjDyrNKq9VL8="/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="71">
+  <si>
+    <t>(HANYA YANG BISA DIATRIBUSIKAN KE ENTITAS INDUK SAJA)</t>
+  </si>
+  <si>
+    <t>ARCI</t>
+  </si>
+  <si>
+    <t>DINYATAKAN DALAM RUPIAH</t>
+  </si>
+  <si>
+    <t>kecuali nilai nominal dan data saham</t>
+  </si>
+  <si>
+    <t>Q2 2026</t>
+  </si>
+  <si>
+    <t>Q1 2026</t>
+  </si>
+  <si>
+    <t>Q4 2025</t>
+  </si>
+  <si>
+    <t>Q3 2025</t>
+  </si>
+  <si>
+    <t>Q2 2025</t>
+  </si>
+  <si>
+    <t>Q1 2025</t>
+  </si>
+  <si>
+    <t>TAHUNAN 2024</t>
+  </si>
+  <si>
+    <t>Q3 2024</t>
+  </si>
+  <si>
+    <t>Q2 2024</t>
+  </si>
+  <si>
+    <t>Q1 2024</t>
+  </si>
+  <si>
+    <t>TAHUNAN 2023</t>
+  </si>
+  <si>
+    <t>Q3 2023</t>
+  </si>
+  <si>
+    <t>Q2 2023</t>
+  </si>
+  <si>
+    <t>Q1 2023</t>
+  </si>
+  <si>
+    <t>TAHUNAN 2022</t>
+  </si>
+  <si>
+    <t>Q3 2022</t>
+  </si>
+  <si>
+    <t>Q2 2022</t>
+  </si>
+  <si>
+    <t>Q1 2022</t>
+  </si>
+  <si>
+    <t>TAHUNAN 2021</t>
+  </si>
+  <si>
+    <t>Q3 2021</t>
+  </si>
+  <si>
+    <t>Q2 2021</t>
+  </si>
+  <si>
+    <t>Q1 2021</t>
+  </si>
+  <si>
+    <t>TAHUNAN 2020</t>
+  </si>
+  <si>
+    <t>Q3 2020</t>
+  </si>
+  <si>
+    <t>Q2 2020</t>
+  </si>
+  <si>
+    <t>Q1 2020</t>
+  </si>
+  <si>
+    <t>Aset</t>
+  </si>
+  <si>
+    <t>total aset lancar</t>
+  </si>
+  <si>
+    <t>KAS</t>
+  </si>
+  <si>
+    <t>liabilitas</t>
+  </si>
+  <si>
+    <t>Utang Bank SAJA Jangka Pendek + Panjang jatuh tempo</t>
+  </si>
+  <si>
+    <t>ekuitas</t>
+  </si>
+  <si>
+    <t>laba bersih</t>
+  </si>
+  <si>
+    <t>pendapatan dari kontrak dengan pelanggan</t>
+  </si>
+  <si>
+    <t>kas dari aktivitas operasi</t>
+  </si>
+  <si>
+    <t>total share</t>
+  </si>
+  <si>
+    <t>Harga saham rupiah</t>
+  </si>
+  <si>
+    <t>Book Value per share</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>ROA</t>
+  </si>
+  <si>
+    <t>ROE</t>
+  </si>
+  <si>
+    <t>PBV</t>
+  </si>
+  <si>
+    <t>PE</t>
+  </si>
+  <si>
+    <t>EPS</t>
+  </si>
+  <si>
+    <t>DER</t>
+  </si>
+  <si>
+    <t>Kurs</t>
+  </si>
+  <si>
+    <t>USD to IDR</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Converted</t>
+  </si>
   <si>
     <t>Perusahaan</t>
   </si>
   <si>
-    <t>(HANYA YANG BISA DIATRIBUSIKAN KE ENTITAS INDUK SAJA)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lokasi </t>
   </si>
   <si>
@@ -117,165 +248,6 @@
   </si>
   <si>
     <t>Tanjung Buyu Perkasa Plantation</t>
-  </si>
-  <si>
-    <t>DINYATAKAN DALAM RUPIAH</t>
-  </si>
-  <si>
-    <t>kecuali nilai nominal dan data saham</t>
-  </si>
-  <si>
-    <t>Q2 2026</t>
-  </si>
-  <si>
-    <t>Q1 2026</t>
-  </si>
-  <si>
-    <t>Q4 2025</t>
-  </si>
-  <si>
-    <t>Q3 2025</t>
-  </si>
-  <si>
-    <t>Q2 2025</t>
-  </si>
-  <si>
-    <t>Q1 2025</t>
-  </si>
-  <si>
-    <t>TAHUNAN 2024</t>
-  </si>
-  <si>
-    <t>Q3 2024</t>
-  </si>
-  <si>
-    <t>Q2 2024</t>
-  </si>
-  <si>
-    <t>Q1 2024</t>
-  </si>
-  <si>
-    <t>TAHUNAN 2023</t>
-  </si>
-  <si>
-    <t>Q3 2023</t>
-  </si>
-  <si>
-    <t>Q2 2023</t>
-  </si>
-  <si>
-    <t>Q1 2023</t>
-  </si>
-  <si>
-    <t>TAHUNAN 2022</t>
-  </si>
-  <si>
-    <t>Q3 2022</t>
-  </si>
-  <si>
-    <t>Q2 2022</t>
-  </si>
-  <si>
-    <t>Q1 2022</t>
-  </si>
-  <si>
-    <t>TAHUNAN 2021</t>
-  </si>
-  <si>
-    <t>Q3 2021</t>
-  </si>
-  <si>
-    <t>Q2 2021</t>
-  </si>
-  <si>
-    <t>Q1 2021</t>
-  </si>
-  <si>
-    <t>TAHUNAN 2020</t>
-  </si>
-  <si>
-    <t>Q3 2020</t>
-  </si>
-  <si>
-    <t>Q2 2020</t>
-  </si>
-  <si>
-    <t>Q1 2020</t>
-  </si>
-  <si>
-    <t>Aset</t>
-  </si>
-  <si>
-    <t>total aset lancar</t>
-  </si>
-  <si>
-    <t>KAS</t>
-  </si>
-  <si>
-    <t>liabilitas</t>
-  </si>
-  <si>
-    <t>Utang Bank SAJA Jangka Pendek + Panjang jatuh tempo</t>
-  </si>
-  <si>
-    <t>ekuitas</t>
-  </si>
-  <si>
-    <t>laba bersih</t>
-  </si>
-  <si>
-    <t>pendapatan dari kontrak dengan pelanggan</t>
-  </si>
-  <si>
-    <t>kas dari aktivitas operasi</t>
-  </si>
-  <si>
-    <t>total share</t>
-  </si>
-  <si>
-    <t>Harga saham rupiah</t>
-  </si>
-  <si>
-    <t>Book Value per share</t>
-  </si>
-  <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>ROA</t>
-  </si>
-  <si>
-    <t>ROE</t>
-  </si>
-  <si>
-    <t>PBV</t>
-  </si>
-  <si>
-    <t>PE</t>
-  </si>
-  <si>
-    <t>EPS</t>
-  </si>
-  <si>
-    <t>DER</t>
-  </si>
-  <si>
-    <t>ARCI</t>
-  </si>
-  <si>
-    <t>Kurs</t>
-  </si>
-  <si>
-    <t>USD to IDR</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Converted</t>
-  </si>
-  <si>
-    <t>25235000000.0</t>
   </si>
 </sst>
 </file>
@@ -363,7 +335,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -621,13 +593,9 @@
     <col min="3" max="3" width="19.5" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="7" width="19.5" customWidth="1"/>
-    <col min="8" max="8" width="17.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.5" customWidth="1"/>
-    <col min="10" max="10" width="17.5" customWidth="1"/>
-    <col min="11" max="11" width="17.1640625" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="8.6640625" customWidth="1"/>
-    <col min="15" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -639,10 +607,10 @@
   <sheetData>
     <row r="1" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="12" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>66</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -669,12 +637,12 @@
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -700,87 +668,87 @@
     <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="S3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="T3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="U3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="V3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="W3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="X3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="Y3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="Z3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="AA3" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="T3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="V3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="W3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y3" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA3" s="6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5">
         <v>19189496535714</v>
@@ -825,13 +793,13 @@
         <v>11020926611446</v>
       </c>
       <c r="P4" s="5">
-        <v>11286421729559.748</v>
+        <v>11286421729559.75</v>
       </c>
       <c r="Q4" s="5">
-        <v>11028397774390.242</v>
+        <v>11028397774390.24</v>
       </c>
       <c r="R4" s="5">
-        <v>10560298900445.766</v>
+        <v>10560298900445.77</v>
       </c>
       <c r="S4" s="5">
         <v>9966590200860.832</v>
@@ -847,7 +815,7 @@
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B5" s="5">
         <v>2979297232143</v>
@@ -892,16 +860,16 @@
         <v>1191006762048</v>
       </c>
       <c r="P5" s="5">
-        <v>1370668490566.0376</v>
+        <v>1370668490566.0381</v>
       </c>
       <c r="Q5" s="5">
-        <v>1142124496951.2195</v>
+        <v>1142124496951.219</v>
       </c>
       <c r="R5" s="5">
-        <v>1296301263001.4858</v>
+        <v>1296301263001.4861</v>
       </c>
       <c r="S5" s="5">
-        <v>1052012410329.9857</v>
+        <v>1052012410329.986</v>
       </c>
       <c r="T5" s="5"/>
       <c r="U5" s="7"/>
@@ -914,7 +882,7 @@
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B6" s="5">
         <v>409296625000</v>
@@ -959,16 +927,16 @@
         <v>95256641566</v>
       </c>
       <c r="P6" s="5">
-        <v>162569716981.13208</v>
+        <v>162569716981.13211</v>
       </c>
       <c r="Q6" s="5">
-        <v>146141859756.09753</v>
+        <v>146141859756.0975</v>
       </c>
       <c r="R6" s="17">
         <v>184978038633</v>
       </c>
       <c r="S6" s="5">
-        <v>331786255380.20087</v>
+        <v>331786255380.20093</v>
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="7"/>
@@ -981,7 +949,7 @@
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B7" s="5">
         <v>11803092071429</v>
@@ -1048,7 +1016,7 @@
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B8" s="5">
         <v>1090018553571</v>
@@ -1096,13 +1064,13 @@
         <v>1503778443396</v>
       </c>
       <c r="Q8" s="5">
-        <v>1221905746951.2192</v>
+        <v>1221905746951.219</v>
       </c>
       <c r="R8" s="5">
         <v>959718053491.82776</v>
       </c>
       <c r="S8" s="5">
-        <v>1468543529411.7646</v>
+        <v>1468543529411.7649</v>
       </c>
       <c r="T8" s="5"/>
       <c r="U8" s="7"/>
@@ -1115,7 +1083,7 @@
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="B9" s="5">
         <v>7353328160714</v>
@@ -1163,13 +1131,13 @@
         <v>3896822720126</v>
       </c>
       <c r="Q9" s="5">
-        <v>3782433124999.9995</v>
+        <v>3782433125000</v>
       </c>
       <c r="R9" s="13">
         <v>3670567132243.6851</v>
       </c>
       <c r="S9" s="5">
-        <v>3475782496413.1997</v>
+        <v>3475782496413.2002</v>
       </c>
       <c r="T9" s="5"/>
       <c r="U9" s="7"/>
@@ -1182,7 +1150,7 @@
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B10" s="5">
         <v>1433061178571</v>
@@ -1230,13 +1198,13 @@
         <v>228784339623</v>
       </c>
       <c r="Q10" s="5">
-        <v>231810807926.82925</v>
+        <v>231810807926.82932</v>
       </c>
       <c r="R10" s="5">
         <v>210274992570.5795</v>
       </c>
       <c r="S10" s="5">
-        <v>135587948350.07175</v>
+        <v>135587948350.0717</v>
       </c>
       <c r="T10" s="5"/>
       <c r="U10" s="7"/>
@@ -1249,7 +1217,7 @@
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="B11" s="5">
         <v>5755149375000</v>
@@ -1297,13 +1265,13 @@
         <v>3403714968553</v>
       </c>
       <c r="Q11" s="5">
-        <v>2525081006097.5605</v>
+        <v>2525081006097.561</v>
       </c>
       <c r="R11" s="5">
-        <v>1777560772659.7327</v>
+        <v>1777560772659.7329</v>
       </c>
       <c r="S11" s="5">
-        <v>1149631348637.0159</v>
+        <v>1149631348637.0161</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="7"/>
@@ -1316,7 +1284,7 @@
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="B12" s="5">
         <v>1645245910714</v>
@@ -1367,10 +1335,10 @@
         <v>560685746951.21948</v>
       </c>
       <c r="R12" s="5">
-        <v>247243491827.63745</v>
+        <v>247243491827.63751</v>
       </c>
       <c r="S12" s="5">
-        <v>522079942611.19086</v>
+        <v>522079942611.19092</v>
       </c>
       <c r="T12" s="5"/>
       <c r="U12" s="7"/>
@@ -1383,7 +1351,7 @@
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="B13" s="5">
         <v>25235000000</v>
@@ -1450,38 +1418,70 @@
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1225</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1110</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1410</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1190</v>
+      </c>
+      <c r="F14" s="4">
+        <v>665</v>
+      </c>
+      <c r="G14" s="4">
+        <v>545</v>
+      </c>
+      <c r="H14" s="5">
+        <v>344</v>
+      </c>
+      <c r="I14" s="5">
+        <v>262</v>
+      </c>
+      <c r="J14" s="5">
+        <v>292</v>
+      </c>
+      <c r="K14" s="5">
+        <v>258</v>
+      </c>
+      <c r="L14" s="5">
+        <v>302</v>
+      </c>
+      <c r="M14" s="5">
+        <v>354</v>
+      </c>
+      <c r="N14" s="5">
+        <v>372</v>
+      </c>
+      <c r="O14" s="5">
+        <v>334</v>
+      </c>
+      <c r="P14" s="5">
+        <v>336</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>340</v>
+      </c>
       <c r="R14" s="5">
-        <v>610</v>
+        <v>366</v>
       </c>
       <c r="S14" s="5">
         <v>352</v>
       </c>
       <c r="T14" s="5">
-        <v>725</v>
+        <v>394</v>
       </c>
       <c r="U14" s="7">
-        <v>570</v>
+        <v>600</v>
       </c>
       <c r="V14" s="7">
-        <v>570</v>
+        <v>590</v>
       </c>
       <c r="W14" s="4">
         <v>570</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="B15" s="6">
         <f t="shared" ref="B15:AA15" si="0">B9/B13</f>
@@ -1540,7 +1540,7 @@
         <v>170.59892631266359</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" si="0"/>
+        <f>K9/K13</f>
         <v>164.70837735075497</v>
       </c>
       <c r="L15" s="6">
@@ -1572,8 +1572,8 @@
         <v>147.79815310020879</v>
       </c>
       <c r="S15" s="6">
-        <f>S9/S13</f>
-        <v>139.95500287550632</v>
+        <f t="shared" si="0"/>
+        <v>139.95500287550635</v>
       </c>
       <c r="T15" s="6" t="e">
         <f t="shared" si="0"/>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B16" s="6">
         <f t="shared" ref="B16:AA16" si="1">B5-B7</f>
@@ -1670,19 +1670,19 @@
       </c>
       <c r="P16" s="6">
         <f t="shared" si="1"/>
-        <v>-6020227468552.9629</v>
+        <v>-6020227468552.9619</v>
       </c>
       <c r="Q16" s="6">
         <f t="shared" si="1"/>
-        <v>-6106053353658.5352</v>
+        <v>-6106053353658.5361</v>
       </c>
       <c r="R16" s="6">
         <f t="shared" si="1"/>
         <v>-5595913655274.8887</v>
       </c>
       <c r="S16" s="6">
-        <f>S5-S7</f>
-        <v>-5439896183644.1904</v>
+        <f t="shared" si="1"/>
+        <v>-5439896183644.1895</v>
       </c>
       <c r="T16" s="6">
         <f t="shared" si="1"/>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="17" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="B17" s="10">
         <f t="shared" ref="B17:AA17" si="2">B10/B4</f>
@@ -1779,19 +1779,19 @@
       </c>
       <c r="P17" s="10">
         <f t="shared" si="2"/>
-        <v>2.0270759422696519E-2</v>
+        <v>2.0270759422696516E-2</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="2"/>
-        <v>2.1019445677334214E-2</v>
+        <v>2.1019445677334225E-2</v>
       </c>
       <c r="R17" s="10">
         <f t="shared" si="2"/>
-        <v>1.9911840995495259E-2</v>
+        <v>1.9911840995495252E-2</v>
       </c>
       <c r="S17" s="10">
         <f t="shared" si="2"/>
-        <v>1.3604246348802499E-2</v>
+        <v>1.3604246348802496E-2</v>
       </c>
       <c r="T17" s="10" t="e">
         <f t="shared" si="2"/>
@@ -1828,7 +1828,7 @@
     </row>
     <row r="18" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="B18" s="10">
         <f t="shared" ref="B18:AA18" si="3">B10/B9</f>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="Q18" s="10">
         <f t="shared" si="3"/>
-        <v>6.1286161649409011E-2</v>
+        <v>6.1286161649409018E-2</v>
       </c>
       <c r="R18" s="10">
         <f t="shared" si="3"/>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="S18" s="10">
         <f t="shared" si="3"/>
-        <v>3.9009330557936359E-2</v>
+        <v>3.9009330557936338E-2</v>
       </c>
       <c r="T18" s="10" t="e">
         <f t="shared" si="3"/>
@@ -1937,79 +1937,79 @@
     </row>
     <row r="19" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:AA19" si="4">B14/B15</f>
-        <v>0</v>
+        <v>4.2039297477780986</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4.2036681449640145</v>
       </c>
       <c r="D19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5.8550666239364846</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5.1652338927827683</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3.3046583172132777</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.8835577788643629</v>
       </c>
       <c r="H19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.9377607195649673</v>
       </c>
       <c r="I19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.6617059067025786</v>
       </c>
       <c r="J19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.7116168683549609</v>
       </c>
       <c r="K19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.5664048432131397</v>
       </c>
       <c r="L19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.8540812402465809</v>
       </c>
       <c r="M19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.1821781845305726</v>
       </c>
       <c r="N19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.4043311904406472</v>
       </c>
       <c r="O19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.1760920475265255</v>
       </c>
       <c r="P19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.1413753201814085</v>
       </c>
       <c r="Q19" s="11">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.2323990196125414</v>
       </c>
       <c r="R19" s="11">
         <f t="shared" si="4"/>
-        <v>4.1272504913265946</v>
+        <v>2.4763502947959566</v>
       </c>
       <c r="S19" s="11">
         <f t="shared" si="4"/>
-        <v>2.5150940857263482</v>
+        <v>2.5150940857263477</v>
       </c>
       <c r="T19" s="11" t="e">
         <f t="shared" si="4"/>
@@ -2046,79 +2046,79 @@
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B20" s="11">
         <f t="shared" ref="B20:AA20" si="5">B14/B21</f>
-        <v>0</v>
+        <v>21.571217936993641</v>
       </c>
       <c r="C20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>55.282154516360258</v>
       </c>
       <c r="D20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>20.827217020883477</v>
       </c>
       <c r="E20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>25.160002749806161</v>
       </c>
       <c r="F20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>29.173630313321112</v>
       </c>
       <c r="G20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>79.35522743102986</v>
       </c>
       <c r="H20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>50.568378583524932</v>
       </c>
       <c r="I20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-110.43256051422692</v>
       </c>
       <c r="J20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-113.60252528951516</v>
       </c>
       <c r="K20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-96.637604232597525</v>
       </c>
       <c r="L20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>33.40904274268113</v>
       </c>
       <c r="M20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>51.821168592735773</v>
       </c>
       <c r="N20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>84.21786386099771</v>
       </c>
       <c r="O20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>113.58745726200851</v>
       </c>
       <c r="P20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>36.473475473673155</v>
       </c>
       <c r="Q20" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>36.425825333671682</v>
       </c>
       <c r="R20" s="11">
         <f t="shared" si="5"/>
-        <v>72.045419261708318</v>
+        <v>43.227251557024985</v>
       </c>
       <c r="S20" s="11">
         <f t="shared" si="5"/>
-        <v>64.47416681480729</v>
+        <v>64.474166814807305</v>
       </c>
       <c r="T20" s="11" t="e">
         <f t="shared" si="5"/>
@@ -2155,7 +2155,7 @@
     </row>
     <row r="21" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B21" s="6">
         <f t="shared" ref="B21:AA21" si="6">B10/B13</f>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="Q21" s="6">
         <f t="shared" si="6"/>
-        <v>9.3340369610158742</v>
+        <v>9.3340369610158778</v>
       </c>
       <c r="R21" s="6">
         <f t="shared" si="6"/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="S21" s="6">
         <f t="shared" si="6"/>
-        <v>5.4595509704075598</v>
+        <v>5.459550970407558</v>
       </c>
       <c r="T21" s="6" t="e">
         <f t="shared" si="6"/>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="22" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="B22" s="10">
         <f t="shared" ref="B22:AA22" si="7">B7/B9</f>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="Q22" s="10">
         <f t="shared" si="7"/>
-        <v>1.9162738933050549</v>
+        <v>1.9162738933050547</v>
       </c>
       <c r="R22" s="10">
         <f t="shared" si="7"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="S22" s="10">
         <f t="shared" si="7"/>
-        <v>1.8677545561822233</v>
+        <v>1.8677545561822231</v>
       </c>
       <c r="T22" s="10" t="e">
         <f t="shared" si="7"/>
@@ -2374,101 +2374,40 @@
     <row r="23" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="25" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D25" s="18">
-        <v>19189496535714</v>
-      </c>
-      <c r="E25" s="18">
-        <v>2979297232143</v>
-      </c>
-      <c r="F25" s="18">
-        <v>409296625000</v>
-      </c>
-      <c r="G25" s="18">
-        <v>11803092071429</v>
-      </c>
-      <c r="H25" s="18">
-        <v>1090018553571</v>
-      </c>
-      <c r="I25" s="18">
-        <v>7353328160714</v>
-      </c>
-      <c r="J25" s="18">
-        <v>1433061178571</v>
-      </c>
-      <c r="K25" s="18">
-        <v>5755149375000</v>
-      </c>
-      <c r="L25" s="18">
-        <v>1645245910714</v>
-      </c>
-      <c r="M25" s="18" t="s">
-        <v>71</v>
-      </c>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="18"/>
     </row>
     <row r="26" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D27" cm="1">
-        <f t="array" ref="D27:D36">TRANSPOSE(D25:M25)</f>
-        <v>19189496535714</v>
-      </c>
-    </row>
-    <row r="28" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D28">
-        <v>2979297232143</v>
-      </c>
-    </row>
-    <row r="29" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D29">
-        <v>409296625000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D30">
-        <v>11803092071429</v>
-      </c>
-    </row>
-    <row r="31" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D31">
-        <v>1090018553571</v>
-      </c>
-    </row>
-    <row r="32" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D32">
-        <v>7353328160714</v>
-      </c>
-    </row>
-    <row r="33" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D33">
-        <v>1433061178571</v>
-      </c>
-    </row>
-    <row r="34" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D34">
-        <v>5755149375000</v>
-      </c>
-    </row>
-    <row r="35" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D35">
-        <v>1645245910714</v>
-      </c>
-    </row>
-    <row r="36" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D36" t="str">
-        <v>25235000000.0</v>
-      </c>
-    </row>
-    <row r="37" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="4:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3428,7 +3367,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB258A72-9464-5845-A57C-12441F1547AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3440,16 +3379,16 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C1" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -3484,7 +3423,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -3498,142 +3437,142 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="C2" s="1">
         <v>3734</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="C3" s="1">
         <v>6365</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="C4" s="3">
         <v>6267</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C5" s="3">
         <v>5029</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C6" s="3">
         <v>10794</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C7" s="3">
         <v>3356</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C8" s="3">
         <v>16348</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="C9" s="3">
         <v>1528</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="C10" s="3">
         <v>11009</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: add more ground truth for the evaluation
</commit_message>
<xml_diff>
--- a/data/ground_truth/ARCI.xlsx
+++ b/data/ground_truth/ARCI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadnajmirahmani/Belajar/ProjectDatasaur/data/ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A571F0D3-469A-BA45-939B-3809BBF92057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0458C743-5B2E-D14A-8751-6175D6C1B91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29300" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -337,7 +337,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -369,6 +369,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
@@ -750,46 +751,46 @@
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="19">
         <v>19189496535714</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="19">
         <v>18047481428571</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="19">
         <v>17227573439597</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="19">
         <v>15886383333333</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="19">
         <v>14580815081169</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="19">
         <v>14619914494196</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="19">
         <v>13980610613893</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="19">
         <v>12766261376702</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="19">
         <v>13503189704433</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="19">
         <v>12882307892235</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="19">
         <v>12381820970724</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="19">
         <v>12334644565217</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="19">
         <v>11325048408408</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="19">
         <v>11020926611446</v>
       </c>
       <c r="P4" s="5">
@@ -817,46 +818,46 @@
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="19">
         <v>2979297232143</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="19">
         <v>2927146258503</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="19">
         <v>2887927147651</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="19">
         <v>2184739283333</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="19">
         <v>1349429951299</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="19">
         <v>1366961492537</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="19">
         <v>1499000096931</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="19">
         <v>1229991785174</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="19">
         <v>1289915648604</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="19">
         <v>1417295277338</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="19">
         <v>1457045855162</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="19">
         <v>1741458509317</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="19">
         <v>973281951952</v>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="19">
         <v>1191006762048</v>
       </c>
       <c r="P5" s="5">
@@ -884,46 +885,46 @@
       <c r="A6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="19">
         <v>409296625000</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="19">
         <v>671137295918</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="19">
         <v>417496359060</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="19">
         <v>390399600000</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="19">
         <v>70624772727</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="19">
         <v>47900281924</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="19">
         <v>73296995153</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="19">
         <v>142554009077</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="19">
         <v>175804548440</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="19">
         <v>54720950872</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="19">
         <v>143608274268</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="19">
         <v>277259378882</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="19">
         <v>56026486486</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="19">
         <v>95256641566</v>
       </c>
       <c r="P6" s="5">
@@ -951,46 +952,46 @@
       <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="19">
         <v>11803092071429</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="19">
         <v>11364988384354</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="19">
         <v>11138182298658</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="19">
         <v>10153818500000</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="19">
         <v>9575570211039</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="19">
         <v>9921723548922</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="19">
         <v>9570979579968</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="19">
         <v>8849227080182</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="19">
         <v>9266104597701</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="19">
         <v>8790164072900</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="19">
         <v>8335133990755</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="19">
         <v>8302537375776</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="19">
         <v>7478349204204</v>
       </c>
-      <c r="O7" s="5">
+      <c r="O7" s="19">
         <v>7212862966867</v>
       </c>
       <c r="P7" s="5">
@@ -1018,46 +1019,46 @@
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="19">
         <v>1090018553571</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="19">
         <v>834453248299</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="19">
         <v>956825738255</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="19">
         <v>1852997600000</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="19">
         <v>1556383457792</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="19">
         <v>1315414726368</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="19">
         <v>1033713780291</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="19">
         <v>789302329803</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="19">
         <v>819519967159</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="19">
         <v>767365721078</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="19">
         <v>757654699538</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="19">
         <v>759932531056</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="19">
         <v>1956975885886</v>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="19">
         <v>1691064608434</v>
       </c>
       <c r="P8" s="5">
@@ -1085,46 +1086,46 @@
       <c r="A9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="19">
         <v>7353328160714</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="19">
         <v>6663430374150</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="19">
         <v>6077018808725</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="19">
         <v>5721647966667</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="19">
         <v>4997574155844</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="19">
         <v>4693880281924</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="19">
         <v>4408820920840</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="19">
         <v>3915716959153</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="19">
         <v>4236824334975</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="19">
         <v>4090532551506</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="19">
         <v>4045221879815</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="19">
         <v>4028813990683</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="19">
         <v>3842490600601</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="19">
         <v>3811828644578</v>
       </c>
       <c r="P9" s="5">
@@ -1152,46 +1153,46 @@
       <c r="A10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="19">
         <v>1433061178571</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="19">
         <v>506688826531</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="19">
         <v>1708406359060</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="19">
         <v>1174628250000</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="19">
         <v>566102840909</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="19">
         <v>170563117745</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="19">
         <v>168944313409</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="19">
         <v>-58920756430</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="19">
         <v>-63835024631</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="19">
         <v>-66303692552</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="19">
         <v>224495208012</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="19">
         <v>169652484472</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="19">
         <v>109699054054</v>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="19">
         <v>73026460843</v>
       </c>
       <c r="P10" s="5">
@@ -1219,46 +1220,46 @@
       <c r="A11" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="19">
         <v>5755149375000</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="19">
         <v>2328361428571</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="19">
         <v>8326003741611</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="19">
         <v>5478341016667</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="19">
         <v>3125823311688</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="19">
         <v>1505426948590</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="19">
         <v>4646508513732</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="19">
         <v>3257286263238</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="19">
         <v>2345676732348</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="19">
         <v>903510570523</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="19">
         <v>3846390878274</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="19">
         <v>2675790916149</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="19">
         <v>1732177147147</v>
       </c>
-      <c r="O11" s="5">
+      <c r="O11" s="19">
         <v>851079141566</v>
       </c>
       <c r="P11" s="5">
@@ -1286,46 +1287,46 @@
       <c r="A12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="19">
         <v>1645245910714</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="19">
         <v>827912023810</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="19">
         <v>879448909396</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="19">
         <v>1450888483333</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="19">
         <v>675487191558</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="19">
         <v>355914096186</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="19">
         <v>1454744103393</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="19">
         <v>1002810680787</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="19">
         <v>776953957307</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="19">
         <v>332297448494</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="19">
         <v>327001402157</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="19">
         <v>9790403727</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="19">
         <v>905774459459</v>
       </c>
-      <c r="O12" s="5">
+      <c r="O12" s="19">
         <v>375205030120</v>
       </c>
       <c r="P12" s="5">
@@ -1353,46 +1354,46 @@
       <c r="A13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="19">
         <v>25235000000</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="19">
         <v>25235000000</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="19">
         <v>25235000000</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="L13" s="5">
+      <c r="L13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="M13" s="5">
+      <c r="M13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="N13" s="5">
+      <c r="N13" s="19">
         <v>24835000000</v>
       </c>
-      <c r="O13" s="5">
+      <c r="O13" s="19">
         <v>24835000000</v>
       </c>
       <c r="P13" s="5">
@@ -1421,13 +1422,13 @@
         <v>40</v>
       </c>
       <c r="B14" s="4">
-        <v>1225</v>
+        <v>1320</v>
       </c>
       <c r="C14" s="4">
         <v>1110</v>
       </c>
       <c r="D14" s="4">
-        <v>1410</v>
+        <v>1315</v>
       </c>
       <c r="E14" s="4">
         <v>1190</v>
@@ -1442,13 +1443,13 @@
         <v>344</v>
       </c>
       <c r="I14" s="5">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="J14" s="5">
         <v>292</v>
       </c>
       <c r="K14" s="5">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="L14" s="5">
         <v>302</v>
@@ -1484,7 +1485,7 @@
         <v>590</v>
       </c>
       <c r="W14" s="4">
-        <v>570</v>
+        <v>755</v>
       </c>
       <c r="X14" s="7">
         <v>570</v>
@@ -1540,7 +1541,7 @@
         <v>170.59892631266359</v>
       </c>
       <c r="K15" s="6">
-        <f>K9/K13</f>
+        <f t="shared" si="0"/>
         <v>164.70837735075497</v>
       </c>
       <c r="L15" s="6">
@@ -1941,7 +1942,7 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:AA19" si="4">B14/B15</f>
-        <v>4.2039297477780986</v>
+        <v>4.529948789442523</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="4"/>
@@ -1949,7 +1950,7 @@
       </c>
       <c r="D19" s="11">
         <f t="shared" si="4"/>
-        <v>5.8550666239364846</v>
+        <v>5.4605763194868633</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="4"/>
@@ -1969,7 +1970,7 @@
       </c>
       <c r="I19" s="11">
         <f t="shared" si="4"/>
-        <v>1.6617059067025786</v>
+        <v>1.7124450183576192</v>
       </c>
       <c r="J19" s="11">
         <f t="shared" si="4"/>
@@ -1977,7 +1978,7 @@
       </c>
       <c r="K19" s="11">
         <f t="shared" si="4"/>
-        <v>1.5664048432131397</v>
+        <v>1.4571207843843161</v>
       </c>
       <c r="L19" s="11">
         <f t="shared" si="4"/>
@@ -2050,7 +2051,7 @@
       </c>
       <c r="B20" s="11">
         <f t="shared" ref="B20:AA20" si="5">B14/B21</f>
-        <v>21.571217936993641</v>
+        <v>23.244087899454371</v>
       </c>
       <c r="C20" s="11">
         <f t="shared" si="5"/>
@@ -2058,7 +2059,7 @@
       </c>
       <c r="D20" s="11">
         <f t="shared" si="5"/>
-        <v>20.827217020883477</v>
+        <v>19.423964810256575</v>
       </c>
       <c r="E20" s="11">
         <f t="shared" si="5"/>
@@ -2078,7 +2079,7 @@
       </c>
       <c r="I20" s="11">
         <f t="shared" si="5"/>
-        <v>-110.43256051422692</v>
+        <v>-113.804547094814</v>
       </c>
       <c r="J20" s="11">
         <f t="shared" si="5"/>
@@ -2086,7 +2087,7 @@
       </c>
       <c r="K20" s="11">
         <f t="shared" si="5"/>
-        <v>-96.637604232597525</v>
+        <v>-89.895445797765134</v>
       </c>
       <c r="L20" s="11">
         <f t="shared" si="5"/>

</xml_diff>